<commit_message>
Time tracker closed out for the day — session wrap-up and marketing/client outreach logged, ending at 2.58 hrs total
</commit_message>
<xml_diff>
--- a/outputs/time-tracking/business-activity-time-tracker.xlsx
+++ b/outputs/time-tracking/business-activity-time-tracker.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="56">
   <si>
     <t xml:space="preserve">Business Activity Time Tracker</t>
   </si>
@@ -82,6 +82,12 @@
   </si>
   <si>
     <t xml:space="preserve">Scheduled the 3 LinkedIn drafts (8/17-8/21 batch) via LinkedIn's own scheduler</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Session wrap-up — save my work / commit review</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marketing work — client outreach</t>
   </si>
   <si>
     <t xml:space="preserve">Time Tracking Summary</t>
@@ -748,7 +754,7 @@
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>1.08333333333333</c:v>
+                  <c:v>1.33333333333333</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -766,7 +772,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1</c:v>
+                  <c:v>1.25</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -774,11 +780,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="90249389"/>
-        <c:axId val="8376640"/>
+        <c:axId val="29344632"/>
+        <c:axId val="63416226"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="90249389"/>
+        <c:axId val="29344632"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -811,7 +817,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="8376640"/>
+        <c:crossAx val="63416226"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -819,7 +825,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="8376640"/>
+        <c:axId val="63416226"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -895,7 +901,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="90249389"/>
+        <c:crossAx val="29344632"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1528,26 +1534,46 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9"/>
-      <c r="B12" s="10"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="12" t="str">
+      <c r="A12" s="9" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="E12" s="12" t="n">
         <f aca="false">IF(D12="","",D12/60)</f>
-        <v/>
-      </c>
-      <c r="F12" s="10"/>
+        <v>0.25</v>
+      </c>
+      <c r="F12" s="10" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9"/>
-      <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="12" t="str">
+      <c r="A13" s="9" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D13" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="E13" s="12" t="n">
         <f aca="false">IF(D13="","",D13/60)</f>
-        <v/>
-      </c>
-      <c r="F13" s="10"/>
+        <v>0.25</v>
+      </c>
+      <c r="F13" s="10" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9"/>
@@ -2626,7 +2652,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2636,7 +2662,7 @@
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="13" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B2" s="13"/>
       <c r="C2" s="13"/>
@@ -2646,7 +2672,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B4" s="15" t="n">
         <v>46244</v>
@@ -2654,7 +2680,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B5" s="16" t="n">
         <f aca="false">B4+13</f>
@@ -2663,7 +2689,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B6" s="16" t="n">
         <f aca="true">TODAY()</f>
@@ -2672,7 +2698,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B7" s="17" t="n">
         <f aca="false">MAX(B5-B6,0)</f>
@@ -2681,10 +2707,10 @@
     </row>
     <row r="9" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2692,13 +2718,13 @@
         <v>4</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E10" s="19" t="s">
         <v>3</v>
       </c>
       <c r="F10" s="19" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2707,7 +2733,7 @@
       </c>
       <c r="B11" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A11)</f>
-        <v>1.08333333333333</v>
+        <v>1.33333333333333</v>
       </c>
       <c r="E11" s="22" t="n">
         <f aca="false">$B$4</f>
@@ -2715,12 +2741,12 @@
       </c>
       <c r="F11" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$A$7:$A$107,E11)</f>
-        <v>2.08333333333333</v>
+        <v>2.58333333333333</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B12" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A12)</f>
@@ -2737,7 +2763,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B13" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A13)</f>
@@ -2754,7 +2780,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B14" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A14)</f>
@@ -2771,7 +2797,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B15" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A15)</f>
@@ -2788,7 +2814,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="20" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B16" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A16)</f>
@@ -2809,7 +2835,7 @@
       </c>
       <c r="B17" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A17)</f>
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="E17" s="22" t="n">
         <f aca="false">E16+1</f>
@@ -2822,11 +2848,11 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="23" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B18" s="24" t="n">
         <f aca="false">SUM(B11:B17)</f>
-        <v>2.08333333333333</v>
+        <v>2.58333333333333</v>
       </c>
       <c r="E18" s="22" t="n">
         <f aca="false">E17+1</f>
@@ -2849,7 +2875,7 @@
     </row>
     <row r="20" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="18" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E20" s="22" t="n">
         <f aca="false">E19+1</f>
@@ -2865,10 +2891,10 @@
         <v>5</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E21" s="22" t="n">
         <f aca="false">E20+1</f>
@@ -2901,7 +2927,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B23" s="20" t="s">
         <v>9</v>
@@ -2941,7 +2967,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="20" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B25" s="20" t="s">
         <v>9</v>
@@ -2953,10 +2979,10 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="20" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C26" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A26)</f>
@@ -2965,10 +2991,10 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="20" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B27" s="20" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C27" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A27)</f>
@@ -2977,10 +3003,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="20" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C28" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A28)</f>
@@ -2989,10 +3015,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="20" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C29" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A29)</f>
@@ -3001,10 +3027,10 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="20" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B30" s="20" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C30" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A30)</f>
@@ -3013,10 +3039,10 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="20" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B31" s="20" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C31" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A31)</f>
@@ -3025,10 +3051,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="20" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B32" s="20" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C32" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A32)</f>
@@ -3037,10 +3063,10 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="20" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B33" s="20" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C33" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A33)</f>
@@ -3049,10 +3075,10 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="20" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C34" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A34)</f>
@@ -3061,10 +3087,10 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="20" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B35" s="20" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C35" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A35)</f>
@@ -3073,10 +3099,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="20" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B36" s="20" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C36" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A36)</f>
@@ -3085,10 +3111,10 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="20" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B37" s="20" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C37" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A37)</f>
@@ -3104,7 +3130,7 @@
       </c>
       <c r="C38" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A38)</f>
-        <v>1</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3116,7 +3142,7 @@
       </c>
       <c r="C39" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A39)</f>
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>
@@ -3150,7 +3176,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B1" s="25"/>
       <c r="C1" s="25"/>
@@ -3160,7 +3186,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="26" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B2" s="26"/>
       <c r="C2" s="26"/>
@@ -3173,7 +3199,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="27" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3189,10 +3215,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C6" s="20" t="s">
         <v>9</v>
@@ -3200,7 +3226,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B7" s="20" t="s">
         <v>10</v>
@@ -3211,10 +3237,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C8" s="20" t="s">
         <v>9</v>
@@ -3222,24 +3248,24 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B9" s="20" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C9" s="20" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C10" s="20" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3247,82 +3273,82 @@
         <v>14</v>
       </c>
       <c r="B11" s="20" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C11" s="20" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="20" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C12" s="20" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="20" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C13" s="20" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="20" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C14" s="20" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="20" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C15" s="20" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="20" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C16" s="20" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="20" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C17" s="20" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="20" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C18" s="20" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="20" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C19" s="20" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="20" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C20" s="20" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Blog content built end-to-end for the monthly SEO planning session — keyword data refreshed (a real finding: 4 turnover queries already rank #1), full article drafted and voice-scrubbed with metadata, AI-search structure applied; Day A strength session — printable recommendation sheet built from real prior numbers, then real session logged with progress across the board
</commit_message>
<xml_diff>
--- a/outputs/time-tracking/business-activity-time-tracker.xlsx
+++ b/outputs/time-tracking/business-activity-time-tracker.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="58">
   <si>
     <t xml:space="preserve">Business Activity Time Tracker</t>
   </si>
@@ -88,6 +88,12 @@
   </si>
   <si>
     <t xml:space="preserve">Marketing work — client outreach</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Business development work — automation schedule review, cloud routine cleanup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Business development work — blog content build and keyword research</t>
   </si>
   <si>
     <t xml:space="preserve">Time Tracking Summary</t>
@@ -772,7 +778,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.25</c:v>
+                  <c:v>2.05</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -780,11 +786,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="29344632"/>
-        <c:axId val="63416226"/>
+        <c:axId val="68157697"/>
+        <c:axId val="383251"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="29344632"/>
+        <c:axId val="68157697"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -817,7 +823,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="63416226"/>
+        <c:crossAx val="383251"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -825,7 +831,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="63416226"/>
+        <c:axId val="383251"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -901,7 +907,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="29344632"/>
+        <c:crossAx val="68157697"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1576,26 +1582,46 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9"/>
-      <c r="B14" s="10"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="12" t="str">
+      <c r="A14" s="9" t="n">
+        <v>46245</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <v>23</v>
+      </c>
+      <c r="E14" s="12" t="n">
         <f aca="false">IF(D14="","",D14/60)</f>
-        <v/>
-      </c>
-      <c r="F14" s="10"/>
+        <v>0.383333333333333</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="12" t="str">
+      <c r="A15" s="9" t="n">
+        <v>46245</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D15" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="E15" s="12" t="n">
         <f aca="false">IF(D15="","",D15/60)</f>
-        <v/>
-      </c>
-      <c r="F15" s="10"/>
+        <v>0.416666666666667</v>
+      </c>
+      <c r="F15" s="10" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9"/>
@@ -2652,7 +2678,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2662,7 +2688,7 @@
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B2" s="13"/>
       <c r="C2" s="13"/>
@@ -2672,7 +2698,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B4" s="15" t="n">
         <v>46244</v>
@@ -2680,7 +2706,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B5" s="16" t="n">
         <f aca="false">B4+13</f>
@@ -2689,28 +2715,28 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B6" s="16" t="n">
         <f aca="true">TODAY()</f>
-        <v>46244</v>
+        <v>46245</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B7" s="17" t="n">
         <f aca="false">MAX(B5-B6,0)</f>
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2718,13 +2744,13 @@
         <v>4</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E10" s="19" t="s">
         <v>3</v>
       </c>
       <c r="F10" s="19" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2746,7 +2772,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B12" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A12)</f>
@@ -2758,12 +2784,12 @@
       </c>
       <c r="F12" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$A$7:$A$107,E12)</f>
-        <v>0</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B13" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A13)</f>
@@ -2780,7 +2806,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B14" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A14)</f>
@@ -2797,7 +2823,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B15" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A15)</f>
@@ -2814,7 +2840,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="20" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B16" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A16)</f>
@@ -2835,7 +2861,7 @@
       </c>
       <c r="B17" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A17)</f>
-        <v>1.25</v>
+        <v>2.05</v>
       </c>
       <c r="E17" s="22" t="n">
         <f aca="false">E16+1</f>
@@ -2848,11 +2874,11 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="23" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B18" s="24" t="n">
         <f aca="false">SUM(B11:B17)</f>
-        <v>2.58333333333333</v>
+        <v>3.38333333333333</v>
       </c>
       <c r="E18" s="22" t="n">
         <f aca="false">E17+1</f>
@@ -2875,7 +2901,7 @@
     </row>
     <row r="20" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="18" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E20" s="22" t="n">
         <f aca="false">E19+1</f>
@@ -2891,10 +2917,10 @@
         <v>5</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E21" s="22" t="n">
         <f aca="false">E20+1</f>
@@ -2927,7 +2953,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B23" s="20" t="s">
         <v>9</v>
@@ -2967,7 +2993,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="20" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B25" s="20" t="s">
         <v>9</v>
@@ -2979,10 +3005,10 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="20" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C26" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A26)</f>
@@ -2991,10 +3017,10 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="20" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B27" s="20" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C27" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A27)</f>
@@ -3003,10 +3029,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="20" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C28" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A28)</f>
@@ -3015,10 +3041,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="20" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C29" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A29)</f>
@@ -3027,10 +3053,10 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="20" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B30" s="20" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C30" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A30)</f>
@@ -3039,10 +3065,10 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="20" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B31" s="20" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C31" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A31)</f>
@@ -3051,10 +3077,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="20" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B32" s="20" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C32" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A32)</f>
@@ -3063,10 +3089,10 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="20" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B33" s="20" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C33" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A33)</f>
@@ -3075,10 +3101,10 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="20" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C34" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A34)</f>
@@ -3087,10 +3113,10 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="20" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B35" s="20" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C35" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A35)</f>
@@ -3099,10 +3125,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="20" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B36" s="20" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C36" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A36)</f>
@@ -3111,10 +3137,10 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="20" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B37" s="20" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C37" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A37)</f>
@@ -3130,7 +3156,7 @@
       </c>
       <c r="C38" s="21" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A38)</f>
-        <v>1.25</v>
+        <v>2.05</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3176,7 +3202,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B1" s="25"/>
       <c r="C1" s="25"/>
@@ -3186,7 +3212,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="26" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B2" s="26"/>
       <c r="C2" s="26"/>
@@ -3199,7 +3225,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="27" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3215,10 +3241,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C6" s="20" t="s">
         <v>9</v>
@@ -3226,7 +3252,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B7" s="20" t="s">
         <v>10</v>
@@ -3237,10 +3263,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C8" s="20" t="s">
         <v>9</v>
@@ -3248,24 +3274,24 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B9" s="20" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C9" s="20" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C10" s="20" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3273,82 +3299,82 @@
         <v>14</v>
       </c>
       <c r="B11" s="20" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C11" s="20" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="20" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C12" s="20" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="20" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C13" s="20" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="20" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C14" s="20" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="20" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C15" s="20" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="20" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C16" s="20" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="20" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C17" s="20" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="20" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C18" s="20" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="20" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C19" s="20" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="20" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C20" s="20" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Time tracker logged 2:05 to a new Blog Development subcategory under Marketing; GitHub Desktop untrusted-server warning resolved and push verified against origin; stray Word lock file removed and gitignored
</commit_message>
<xml_diff>
--- a/outputs/time-tracking/business-activity-time-tracker.xlsx
+++ b/outputs/time-tracking/business-activity-time-tracker.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="4"/>
+  <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="60">
   <si>
     <t xml:space="preserve">Business Activity Time Tracker</t>
   </si>
@@ -94,6 +94,12 @@
   </si>
   <si>
     <t xml:space="preserve">Business development work — blog content build and keyword research</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blog Development (Marketing)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blog post review/edit, built out and published in WordPress</t>
   </si>
   <si>
     <t xml:space="preserve">Time Tracking Summary</t>
@@ -433,8 +439,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -474,7 +484,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -490,23 +500,23 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -514,7 +524,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -526,7 +536,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -538,7 +548,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -622,7 +632,6 @@
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
-  <c:style val="10"/>
   <c:chart>
     <c:title>
       <c:tx>
@@ -691,23 +700,27 @@
           <c:invertIfNegative val="0"/>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="outEnd"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
+            <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
             <c:leaderLines>
               <c:spPr>
@@ -760,7 +773,7 @@
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>1.33333333333333</c:v>
+                  <c:v>3.41666666666667</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -786,17 +799,17 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="68157697"/>
-        <c:axId val="383251"/>
+        <c:axId val="8391556"/>
+        <c:axId val="86258886"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="68157697"/>
+        <c:axId val="8391556"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -823,7 +836,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="383251"/>
+        <c:crossAx val="86258886"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -831,7 +844,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="383251"/>
+        <c:axId val="86258886"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -880,7 +893,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -907,7 +920,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="68157697"/>
+        <c:crossAx val="8391556"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1164,9 +1177,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>305640</xdr:colOff>
+      <xdr:colOff>305280</xdr:colOff>
       <xdr:row>40</xdr:row>
-      <xdr:rowOff>22320</xdr:rowOff>
+      <xdr:rowOff>21960</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1174,8 +1187,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="6673320" y="4963320"/>
-        <a:ext cx="5759640" cy="2879640"/>
+        <a:off x="6673320" y="4952880"/>
+        <a:ext cx="5759280" cy="2879640"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1371,1269 +1384,1279 @@
   <dimension ref="A1:F107"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="42"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="n">
         <v>46244</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="7"/>
-      <c r="E7" s="8" t="str">
+      <c r="D7" s="8"/>
+      <c r="E7" s="9" t="str">
         <f aca="false">IF(D7="","",D7/60)</f>
         <v/>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9" t="n">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10" t="n">
         <v>46244</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="11" t="n">
+      <c r="D8" s="12" t="n">
         <v>45</v>
       </c>
-      <c r="E8" s="12" t="n">
+      <c r="E8" s="13" t="n">
         <f aca="false">IF(D8="","",D8/60)</f>
         <v>0.75</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="F8" s="11" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="n">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="10" t="n">
         <v>46244</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="11" t="n">
+      <c r="D9" s="12" t="n">
         <v>60</v>
       </c>
-      <c r="E9" s="12" t="n">
+      <c r="E9" s="13" t="n">
         <f aca="false">IF(D9="","",D9/60)</f>
         <v>1</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="F9" s="11" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9" t="n">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="10" t="n">
         <v>46244</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="11" t="n">
+      <c r="D10" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="E10" s="12" t="n">
+      <c r="E10" s="13" t="n">
         <f aca="false">IF(D10="","",D10/60)</f>
         <v>0.25</v>
       </c>
-      <c r="F10" s="10" t="s">
+      <c r="F10" s="11" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="n">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="10" t="n">
         <v>46244</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="D11" s="11" t="n">
+      <c r="D11" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="E11" s="12" t="n">
+      <c r="E11" s="13" t="n">
         <f aca="false">IF(D11="","",D11/60)</f>
         <v>0.0833333333333333</v>
       </c>
-      <c r="F11" s="10" t="s">
+      <c r="F11" s="11" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9" t="n">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="10" t="n">
         <v>46244</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="11" t="n">
+      <c r="D12" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="E12" s="12" t="n">
+      <c r="E12" s="13" t="n">
         <f aca="false">IF(D12="","",D12/60)</f>
         <v>0.25</v>
       </c>
-      <c r="F12" s="10" t="s">
+      <c r="F12" s="11" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9" t="n">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="10" t="n">
         <v>46244</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="D13" s="11" t="n">
+      <c r="D13" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="E13" s="12" t="n">
+      <c r="E13" s="13" t="n">
         <f aca="false">IF(D13="","",D13/60)</f>
         <v>0.25</v>
       </c>
-      <c r="F13" s="10" t="s">
+      <c r="F13" s="11" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9" t="n">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="n">
         <v>46245</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="D14" s="11" t="n">
+      <c r="D14" s="12" t="n">
         <v>23</v>
       </c>
-      <c r="E14" s="12" t="n">
+      <c r="E14" s="13" t="n">
         <f aca="false">IF(D14="","",D14/60)</f>
         <v>0.383333333333333</v>
       </c>
-      <c r="F14" s="10" t="s">
+      <c r="F14" s="11" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9" t="n">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="n">
         <v>46245</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="D15" s="11" t="n">
+      <c r="D15" s="12" t="n">
         <v>25</v>
       </c>
-      <c r="E15" s="12" t="n">
+      <c r="E15" s="13" t="n">
         <f aca="false">IF(D15="","",D15/60)</f>
         <v>0.416666666666667</v>
       </c>
-      <c r="F15" s="10" t="s">
+      <c r="F15" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9"/>
-      <c r="B16" s="10"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="12" t="str">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="n">
+        <v>46245</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" s="12" t="n">
+        <v>125</v>
+      </c>
+      <c r="E16" s="13" t="n">
         <f aca="false">IF(D16="","",D16/60)</f>
-        <v/>
-      </c>
-      <c r="F16" s="10"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="9"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="12" t="str">
+        <v>2.08333333333333</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="10"/>
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="13" t="str">
         <f aca="false">IF(D17="","",D17/60)</f>
         <v/>
       </c>
-      <c r="F17" s="10"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="9"/>
-      <c r="B18" s="10"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="12" t="str">
+      <c r="F17" s="11"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="10"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="13" t="str">
         <f aca="false">IF(D18="","",D18/60)</f>
         <v/>
       </c>
-      <c r="F18" s="10"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="9"/>
-      <c r="B19" s="10"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="12" t="str">
+      <c r="F18" s="11"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="10"/>
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="13" t="str">
         <f aca="false">IF(D19="","",D19/60)</f>
         <v/>
       </c>
-      <c r="F19" s="10"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="9"/>
-      <c r="B20" s="10"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="12" t="str">
+      <c r="F19" s="11"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="10"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="13" t="str">
         <f aca="false">IF(D20="","",D20/60)</f>
         <v/>
       </c>
-      <c r="F20" s="10"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="9"/>
-      <c r="B21" s="10"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="12" t="str">
+      <c r="F20" s="11"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="10"/>
+      <c r="B21" s="11"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="13" t="str">
         <f aca="false">IF(D21="","",D21/60)</f>
         <v/>
       </c>
-      <c r="F21" s="10"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="9"/>
-      <c r="B22" s="10"/>
-      <c r="C22" s="10"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="12" t="str">
+      <c r="F21" s="11"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="10"/>
+      <c r="B22" s="11"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="13" t="str">
         <f aca="false">IF(D22="","",D22/60)</f>
         <v/>
       </c>
-      <c r="F22" s="10"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="9"/>
-      <c r="B23" s="10"/>
-      <c r="C23" s="10"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="12" t="str">
+      <c r="F22" s="11"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="10"/>
+      <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="13" t="str">
         <f aca="false">IF(D23="","",D23/60)</f>
         <v/>
       </c>
-      <c r="F23" s="10"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="9"/>
-      <c r="B24" s="10"/>
-      <c r="C24" s="10"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="12" t="str">
+      <c r="F23" s="11"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="10"/>
+      <c r="B24" s="11"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="13" t="str">
         <f aca="false">IF(D24="","",D24/60)</f>
         <v/>
       </c>
-      <c r="F24" s="10"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="9"/>
-      <c r="B25" s="10"/>
-      <c r="C25" s="10"/>
-      <c r="D25" s="11"/>
-      <c r="E25" s="12" t="str">
+      <c r="F24" s="11"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="10"/>
+      <c r="B25" s="11"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="12"/>
+      <c r="E25" s="13" t="str">
         <f aca="false">IF(D25="","",D25/60)</f>
         <v/>
       </c>
-      <c r="F25" s="10"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="9"/>
-      <c r="B26" s="10"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="11"/>
-      <c r="E26" s="12" t="str">
+      <c r="F25" s="11"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="10"/>
+      <c r="B26" s="11"/>
+      <c r="C26" s="11"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="13" t="str">
         <f aca="false">IF(D26="","",D26/60)</f>
         <v/>
       </c>
-      <c r="F26" s="10"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="9"/>
-      <c r="B27" s="10"/>
-      <c r="C27" s="10"/>
-      <c r="D27" s="11"/>
-      <c r="E27" s="12" t="str">
+      <c r="F26" s="11"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="10"/>
+      <c r="B27" s="11"/>
+      <c r="C27" s="11"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="13" t="str">
         <f aca="false">IF(D27="","",D27/60)</f>
         <v/>
       </c>
-      <c r="F27" s="10"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="9"/>
-      <c r="B28" s="10"/>
-      <c r="C28" s="10"/>
-      <c r="D28" s="11"/>
-      <c r="E28" s="12" t="str">
+      <c r="F27" s="11"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="10"/>
+      <c r="B28" s="11"/>
+      <c r="C28" s="11"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="13" t="str">
         <f aca="false">IF(D28="","",D28/60)</f>
         <v/>
       </c>
-      <c r="F28" s="10"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="9"/>
-      <c r="B29" s="10"/>
-      <c r="C29" s="10"/>
-      <c r="D29" s="11"/>
-      <c r="E29" s="12" t="str">
+      <c r="F28" s="11"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="10"/>
+      <c r="B29" s="11"/>
+      <c r="C29" s="11"/>
+      <c r="D29" s="12"/>
+      <c r="E29" s="13" t="str">
         <f aca="false">IF(D29="","",D29/60)</f>
         <v/>
       </c>
-      <c r="F29" s="10"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="9"/>
-      <c r="B30" s="10"/>
-      <c r="C30" s="10"/>
-      <c r="D30" s="11"/>
-      <c r="E30" s="12" t="str">
+      <c r="F29" s="11"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="10"/>
+      <c r="B30" s="11"/>
+      <c r="C30" s="11"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="13" t="str">
         <f aca="false">IF(D30="","",D30/60)</f>
         <v/>
       </c>
-      <c r="F30" s="10"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="9"/>
-      <c r="B31" s="10"/>
-      <c r="C31" s="10"/>
-      <c r="D31" s="11"/>
-      <c r="E31" s="12" t="str">
+      <c r="F30" s="11"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="10"/>
+      <c r="B31" s="11"/>
+      <c r="C31" s="11"/>
+      <c r="D31" s="12"/>
+      <c r="E31" s="13" t="str">
         <f aca="false">IF(D31="","",D31/60)</f>
         <v/>
       </c>
-      <c r="F31" s="10"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="9"/>
-      <c r="B32" s="10"/>
-      <c r="C32" s="10"/>
-      <c r="D32" s="11"/>
-      <c r="E32" s="12" t="str">
+      <c r="F31" s="11"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="10"/>
+      <c r="B32" s="11"/>
+      <c r="C32" s="11"/>
+      <c r="D32" s="12"/>
+      <c r="E32" s="13" t="str">
         <f aca="false">IF(D32="","",D32/60)</f>
         <v/>
       </c>
-      <c r="F32" s="10"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="9"/>
-      <c r="B33" s="10"/>
-      <c r="C33" s="10"/>
-      <c r="D33" s="11"/>
-      <c r="E33" s="12" t="str">
+      <c r="F32" s="11"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="10"/>
+      <c r="B33" s="11"/>
+      <c r="C33" s="11"/>
+      <c r="D33" s="12"/>
+      <c r="E33" s="13" t="str">
         <f aca="false">IF(D33="","",D33/60)</f>
         <v/>
       </c>
-      <c r="F33" s="10"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="9"/>
-      <c r="B34" s="10"/>
-      <c r="C34" s="10"/>
-      <c r="D34" s="11"/>
-      <c r="E34" s="12" t="str">
+      <c r="F33" s="11"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="10"/>
+      <c r="B34" s="11"/>
+      <c r="C34" s="11"/>
+      <c r="D34" s="12"/>
+      <c r="E34" s="13" t="str">
         <f aca="false">IF(D34="","",D34/60)</f>
         <v/>
       </c>
-      <c r="F34" s="10"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="9"/>
-      <c r="B35" s="10"/>
-      <c r="C35" s="10"/>
-      <c r="D35" s="11"/>
-      <c r="E35" s="12" t="str">
+      <c r="F34" s="11"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="10"/>
+      <c r="B35" s="11"/>
+      <c r="C35" s="11"/>
+      <c r="D35" s="12"/>
+      <c r="E35" s="13" t="str">
         <f aca="false">IF(D35="","",D35/60)</f>
         <v/>
       </c>
-      <c r="F35" s="10"/>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="9"/>
-      <c r="B36" s="10"/>
-      <c r="C36" s="10"/>
-      <c r="D36" s="11"/>
-      <c r="E36" s="12" t="str">
+      <c r="F35" s="11"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="10"/>
+      <c r="B36" s="11"/>
+      <c r="C36" s="11"/>
+      <c r="D36" s="12"/>
+      <c r="E36" s="13" t="str">
         <f aca="false">IF(D36="","",D36/60)</f>
         <v/>
       </c>
-      <c r="F36" s="10"/>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="9"/>
-      <c r="B37" s="10"/>
-      <c r="C37" s="10"/>
-      <c r="D37" s="11"/>
-      <c r="E37" s="12" t="str">
+      <c r="F36" s="11"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="10"/>
+      <c r="B37" s="11"/>
+      <c r="C37" s="11"/>
+      <c r="D37" s="12"/>
+      <c r="E37" s="13" t="str">
         <f aca="false">IF(D37="","",D37/60)</f>
         <v/>
       </c>
-      <c r="F37" s="10"/>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="9"/>
-      <c r="B38" s="10"/>
-      <c r="C38" s="10"/>
-      <c r="D38" s="11"/>
-      <c r="E38" s="12" t="str">
+      <c r="F37" s="11"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="10"/>
+      <c r="B38" s="11"/>
+      <c r="C38" s="11"/>
+      <c r="D38" s="12"/>
+      <c r="E38" s="13" t="str">
         <f aca="false">IF(D38="","",D38/60)</f>
         <v/>
       </c>
-      <c r="F38" s="10"/>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="9"/>
-      <c r="B39" s="10"/>
-      <c r="C39" s="10"/>
-      <c r="D39" s="11"/>
-      <c r="E39" s="12" t="str">
+      <c r="F38" s="11"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="10"/>
+      <c r="B39" s="11"/>
+      <c r="C39" s="11"/>
+      <c r="D39" s="12"/>
+      <c r="E39" s="13" t="str">
         <f aca="false">IF(D39="","",D39/60)</f>
         <v/>
       </c>
-      <c r="F39" s="10"/>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="9"/>
-      <c r="B40" s="10"/>
-      <c r="C40" s="10"/>
-      <c r="D40" s="11"/>
-      <c r="E40" s="12" t="str">
+      <c r="F39" s="11"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="10"/>
+      <c r="B40" s="11"/>
+      <c r="C40" s="11"/>
+      <c r="D40" s="12"/>
+      <c r="E40" s="13" t="str">
         <f aca="false">IF(D40="","",D40/60)</f>
         <v/>
       </c>
-      <c r="F40" s="10"/>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="9"/>
-      <c r="B41" s="10"/>
-      <c r="C41" s="10"/>
-      <c r="D41" s="11"/>
-      <c r="E41" s="12" t="str">
+      <c r="F40" s="11"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="10"/>
+      <c r="B41" s="11"/>
+      <c r="C41" s="11"/>
+      <c r="D41" s="12"/>
+      <c r="E41" s="13" t="str">
         <f aca="false">IF(D41="","",D41/60)</f>
         <v/>
       </c>
-      <c r="F41" s="10"/>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="9"/>
-      <c r="B42" s="10"/>
-      <c r="C42" s="10"/>
-      <c r="D42" s="11"/>
-      <c r="E42" s="12" t="str">
+      <c r="F41" s="11"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="10"/>
+      <c r="B42" s="11"/>
+      <c r="C42" s="11"/>
+      <c r="D42" s="12"/>
+      <c r="E42" s="13" t="str">
         <f aca="false">IF(D42="","",D42/60)</f>
         <v/>
       </c>
-      <c r="F42" s="10"/>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="9"/>
-      <c r="B43" s="10"/>
-      <c r="C43" s="10"/>
-      <c r="D43" s="11"/>
-      <c r="E43" s="12" t="str">
+      <c r="F42" s="11"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="10"/>
+      <c r="B43" s="11"/>
+      <c r="C43" s="11"/>
+      <c r="D43" s="12"/>
+      <c r="E43" s="13" t="str">
         <f aca="false">IF(D43="","",D43/60)</f>
         <v/>
       </c>
-      <c r="F43" s="10"/>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="9"/>
-      <c r="B44" s="10"/>
-      <c r="C44" s="10"/>
-      <c r="D44" s="11"/>
-      <c r="E44" s="12" t="str">
+      <c r="F43" s="11"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="10"/>
+      <c r="B44" s="11"/>
+      <c r="C44" s="11"/>
+      <c r="D44" s="12"/>
+      <c r="E44" s="13" t="str">
         <f aca="false">IF(D44="","",D44/60)</f>
         <v/>
       </c>
-      <c r="F44" s="10"/>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="9"/>
-      <c r="B45" s="10"/>
-      <c r="C45" s="10"/>
-      <c r="D45" s="11"/>
-      <c r="E45" s="12" t="str">
+      <c r="F44" s="11"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="10"/>
+      <c r="B45" s="11"/>
+      <c r="C45" s="11"/>
+      <c r="D45" s="12"/>
+      <c r="E45" s="13" t="str">
         <f aca="false">IF(D45="","",D45/60)</f>
         <v/>
       </c>
-      <c r="F45" s="10"/>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="9"/>
-      <c r="B46" s="10"/>
-      <c r="C46" s="10"/>
-      <c r="D46" s="11"/>
-      <c r="E46" s="12" t="str">
+      <c r="F45" s="11"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="10"/>
+      <c r="B46" s="11"/>
+      <c r="C46" s="11"/>
+      <c r="D46" s="12"/>
+      <c r="E46" s="13" t="str">
         <f aca="false">IF(D46="","",D46/60)</f>
         <v/>
       </c>
-      <c r="F46" s="10"/>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="9"/>
-      <c r="B47" s="10"/>
-      <c r="C47" s="10"/>
-      <c r="D47" s="11"/>
-      <c r="E47" s="12" t="str">
+      <c r="F46" s="11"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="10"/>
+      <c r="B47" s="11"/>
+      <c r="C47" s="11"/>
+      <c r="D47" s="12"/>
+      <c r="E47" s="13" t="str">
         <f aca="false">IF(D47="","",D47/60)</f>
         <v/>
       </c>
-      <c r="F47" s="10"/>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="9"/>
-      <c r="B48" s="10"/>
-      <c r="C48" s="10"/>
-      <c r="D48" s="11"/>
-      <c r="E48" s="12" t="str">
+      <c r="F47" s="11"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="10"/>
+      <c r="B48" s="11"/>
+      <c r="C48" s="11"/>
+      <c r="D48" s="12"/>
+      <c r="E48" s="13" t="str">
         <f aca="false">IF(D48="","",D48/60)</f>
         <v/>
       </c>
-      <c r="F48" s="10"/>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="9"/>
-      <c r="B49" s="10"/>
-      <c r="C49" s="10"/>
-      <c r="D49" s="11"/>
-      <c r="E49" s="12" t="str">
+      <c r="F48" s="11"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="10"/>
+      <c r="B49" s="11"/>
+      <c r="C49" s="11"/>
+      <c r="D49" s="12"/>
+      <c r="E49" s="13" t="str">
         <f aca="false">IF(D49="","",D49/60)</f>
         <v/>
       </c>
-      <c r="F49" s="10"/>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="9"/>
-      <c r="B50" s="10"/>
-      <c r="C50" s="10"/>
-      <c r="D50" s="11"/>
-      <c r="E50" s="12" t="str">
+      <c r="F49" s="11"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="10"/>
+      <c r="B50" s="11"/>
+      <c r="C50" s="11"/>
+      <c r="D50" s="12"/>
+      <c r="E50" s="13" t="str">
         <f aca="false">IF(D50="","",D50/60)</f>
         <v/>
       </c>
-      <c r="F50" s="10"/>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="9"/>
-      <c r="B51" s="10"/>
-      <c r="C51" s="10"/>
-      <c r="D51" s="11"/>
-      <c r="E51" s="12" t="str">
+      <c r="F50" s="11"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="10"/>
+      <c r="B51" s="11"/>
+      <c r="C51" s="11"/>
+      <c r="D51" s="12"/>
+      <c r="E51" s="13" t="str">
         <f aca="false">IF(D51="","",D51/60)</f>
         <v/>
       </c>
-      <c r="F51" s="10"/>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="9"/>
-      <c r="B52" s="10"/>
-      <c r="C52" s="10"/>
-      <c r="D52" s="11"/>
-      <c r="E52" s="12" t="str">
+      <c r="F51" s="11"/>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="10"/>
+      <c r="B52" s="11"/>
+      <c r="C52" s="11"/>
+      <c r="D52" s="12"/>
+      <c r="E52" s="13" t="str">
         <f aca="false">IF(D52="","",D52/60)</f>
         <v/>
       </c>
-      <c r="F52" s="10"/>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="9"/>
-      <c r="B53" s="10"/>
-      <c r="C53" s="10"/>
-      <c r="D53" s="11"/>
-      <c r="E53" s="12" t="str">
+      <c r="F52" s="11"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="10"/>
+      <c r="B53" s="11"/>
+      <c r="C53" s="11"/>
+      <c r="D53" s="12"/>
+      <c r="E53" s="13" t="str">
         <f aca="false">IF(D53="","",D53/60)</f>
         <v/>
       </c>
-      <c r="F53" s="10"/>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="9"/>
-      <c r="B54" s="10"/>
-      <c r="C54" s="10"/>
-      <c r="D54" s="11"/>
-      <c r="E54" s="12" t="str">
+      <c r="F53" s="11"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="10"/>
+      <c r="B54" s="11"/>
+      <c r="C54" s="11"/>
+      <c r="D54" s="12"/>
+      <c r="E54" s="13" t="str">
         <f aca="false">IF(D54="","",D54/60)</f>
         <v/>
       </c>
-      <c r="F54" s="10"/>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="9"/>
-      <c r="B55" s="10"/>
-      <c r="C55" s="10"/>
-      <c r="D55" s="11"/>
-      <c r="E55" s="12" t="str">
+      <c r="F54" s="11"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="10"/>
+      <c r="B55" s="11"/>
+      <c r="C55" s="11"/>
+      <c r="D55" s="12"/>
+      <c r="E55" s="13" t="str">
         <f aca="false">IF(D55="","",D55/60)</f>
         <v/>
       </c>
-      <c r="F55" s="10"/>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="9"/>
-      <c r="B56" s="10"/>
-      <c r="C56" s="10"/>
-      <c r="D56" s="11"/>
-      <c r="E56" s="12" t="str">
+      <c r="F55" s="11"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="10"/>
+      <c r="B56" s="11"/>
+      <c r="C56" s="11"/>
+      <c r="D56" s="12"/>
+      <c r="E56" s="13" t="str">
         <f aca="false">IF(D56="","",D56/60)</f>
         <v/>
       </c>
-      <c r="F56" s="10"/>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="9"/>
-      <c r="B57" s="10"/>
-      <c r="C57" s="10"/>
-      <c r="D57" s="11"/>
-      <c r="E57" s="12" t="str">
+      <c r="F56" s="11"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="10"/>
+      <c r="B57" s="11"/>
+      <c r="C57" s="11"/>
+      <c r="D57" s="12"/>
+      <c r="E57" s="13" t="str">
         <f aca="false">IF(D57="","",D57/60)</f>
         <v/>
       </c>
-      <c r="F57" s="10"/>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="9"/>
-      <c r="B58" s="10"/>
-      <c r="C58" s="10"/>
-      <c r="D58" s="11"/>
-      <c r="E58" s="12" t="str">
+      <c r="F57" s="11"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="10"/>
+      <c r="B58" s="11"/>
+      <c r="C58" s="11"/>
+      <c r="D58" s="12"/>
+      <c r="E58" s="13" t="str">
         <f aca="false">IF(D58="","",D58/60)</f>
         <v/>
       </c>
-      <c r="F58" s="10"/>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="9"/>
-      <c r="B59" s="10"/>
-      <c r="C59" s="10"/>
-      <c r="D59" s="11"/>
-      <c r="E59" s="12" t="str">
+      <c r="F58" s="11"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="10"/>
+      <c r="B59" s="11"/>
+      <c r="C59" s="11"/>
+      <c r="D59" s="12"/>
+      <c r="E59" s="13" t="str">
         <f aca="false">IF(D59="","",D59/60)</f>
         <v/>
       </c>
-      <c r="F59" s="10"/>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="9"/>
-      <c r="B60" s="10"/>
-      <c r="C60" s="10"/>
-      <c r="D60" s="11"/>
-      <c r="E60" s="12" t="str">
+      <c r="F59" s="11"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="10"/>
+      <c r="B60" s="11"/>
+      <c r="C60" s="11"/>
+      <c r="D60" s="12"/>
+      <c r="E60" s="13" t="str">
         <f aca="false">IF(D60="","",D60/60)</f>
         <v/>
       </c>
-      <c r="F60" s="10"/>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="9"/>
-      <c r="B61" s="10"/>
-      <c r="C61" s="10"/>
-      <c r="D61" s="11"/>
-      <c r="E61" s="12" t="str">
+      <c r="F60" s="11"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="10"/>
+      <c r="B61" s="11"/>
+      <c r="C61" s="11"/>
+      <c r="D61" s="12"/>
+      <c r="E61" s="13" t="str">
         <f aca="false">IF(D61="","",D61/60)</f>
         <v/>
       </c>
-      <c r="F61" s="10"/>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="9"/>
-      <c r="B62" s="10"/>
-      <c r="C62" s="10"/>
-      <c r="D62" s="11"/>
-      <c r="E62" s="12" t="str">
+      <c r="F61" s="11"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="10"/>
+      <c r="B62" s="11"/>
+      <c r="C62" s="11"/>
+      <c r="D62" s="12"/>
+      <c r="E62" s="13" t="str">
         <f aca="false">IF(D62="","",D62/60)</f>
         <v/>
       </c>
-      <c r="F62" s="10"/>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="9"/>
-      <c r="B63" s="10"/>
-      <c r="C63" s="10"/>
-      <c r="D63" s="11"/>
-      <c r="E63" s="12" t="str">
+      <c r="F62" s="11"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="10"/>
+      <c r="B63" s="11"/>
+      <c r="C63" s="11"/>
+      <c r="D63" s="12"/>
+      <c r="E63" s="13" t="str">
         <f aca="false">IF(D63="","",D63/60)</f>
         <v/>
       </c>
-      <c r="F63" s="10"/>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="9"/>
-      <c r="B64" s="10"/>
-      <c r="C64" s="10"/>
-      <c r="D64" s="11"/>
-      <c r="E64" s="12" t="str">
+      <c r="F63" s="11"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="10"/>
+      <c r="B64" s="11"/>
+      <c r="C64" s="11"/>
+      <c r="D64" s="12"/>
+      <c r="E64" s="13" t="str">
         <f aca="false">IF(D64="","",D64/60)</f>
         <v/>
       </c>
-      <c r="F64" s="10"/>
-    </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="9"/>
-      <c r="B65" s="10"/>
-      <c r="C65" s="10"/>
-      <c r="D65" s="11"/>
-      <c r="E65" s="12" t="str">
+      <c r="F64" s="11"/>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="10"/>
+      <c r="B65" s="11"/>
+      <c r="C65" s="11"/>
+      <c r="D65" s="12"/>
+      <c r="E65" s="13" t="str">
         <f aca="false">IF(D65="","",D65/60)</f>
         <v/>
       </c>
-      <c r="F65" s="10"/>
-    </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="9"/>
-      <c r="B66" s="10"/>
-      <c r="C66" s="10"/>
-      <c r="D66" s="11"/>
-      <c r="E66" s="12" t="str">
+      <c r="F65" s="11"/>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="10"/>
+      <c r="B66" s="11"/>
+      <c r="C66" s="11"/>
+      <c r="D66" s="12"/>
+      <c r="E66" s="13" t="str">
         <f aca="false">IF(D66="","",D66/60)</f>
         <v/>
       </c>
-      <c r="F66" s="10"/>
-    </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="9"/>
-      <c r="B67" s="10"/>
-      <c r="C67" s="10"/>
-      <c r="D67" s="11"/>
-      <c r="E67" s="12" t="str">
+      <c r="F66" s="11"/>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="10"/>
+      <c r="B67" s="11"/>
+      <c r="C67" s="11"/>
+      <c r="D67" s="12"/>
+      <c r="E67" s="13" t="str">
         <f aca="false">IF(D67="","",D67/60)</f>
         <v/>
       </c>
-      <c r="F67" s="10"/>
-    </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="9"/>
-      <c r="B68" s="10"/>
-      <c r="C68" s="10"/>
-      <c r="D68" s="11"/>
-      <c r="E68" s="12" t="str">
+      <c r="F67" s="11"/>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="10"/>
+      <c r="B68" s="11"/>
+      <c r="C68" s="11"/>
+      <c r="D68" s="12"/>
+      <c r="E68" s="13" t="str">
         <f aca="false">IF(D68="","",D68/60)</f>
         <v/>
       </c>
-      <c r="F68" s="10"/>
-    </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="9"/>
-      <c r="B69" s="10"/>
-      <c r="C69" s="10"/>
-      <c r="D69" s="11"/>
-      <c r="E69" s="12" t="str">
+      <c r="F68" s="11"/>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="10"/>
+      <c r="B69" s="11"/>
+      <c r="C69" s="11"/>
+      <c r="D69" s="12"/>
+      <c r="E69" s="13" t="str">
         <f aca="false">IF(D69="","",D69/60)</f>
         <v/>
       </c>
-      <c r="F69" s="10"/>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="9"/>
-      <c r="B70" s="10"/>
-      <c r="C70" s="10"/>
-      <c r="D70" s="11"/>
-      <c r="E70" s="12" t="str">
+      <c r="F69" s="11"/>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="10"/>
+      <c r="B70" s="11"/>
+      <c r="C70" s="11"/>
+      <c r="D70" s="12"/>
+      <c r="E70" s="13" t="str">
         <f aca="false">IF(D70="","",D70/60)</f>
         <v/>
       </c>
-      <c r="F70" s="10"/>
-    </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="9"/>
-      <c r="B71" s="10"/>
-      <c r="C71" s="10"/>
-      <c r="D71" s="11"/>
-      <c r="E71" s="12" t="str">
+      <c r="F70" s="11"/>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A71" s="10"/>
+      <c r="B71" s="11"/>
+      <c r="C71" s="11"/>
+      <c r="D71" s="12"/>
+      <c r="E71" s="13" t="str">
         <f aca="false">IF(D71="","",D71/60)</f>
         <v/>
       </c>
-      <c r="F71" s="10"/>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="9"/>
-      <c r="B72" s="10"/>
-      <c r="C72" s="10"/>
-      <c r="D72" s="11"/>
-      <c r="E72" s="12" t="str">
+      <c r="F71" s="11"/>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="10"/>
+      <c r="B72" s="11"/>
+      <c r="C72" s="11"/>
+      <c r="D72" s="12"/>
+      <c r="E72" s="13" t="str">
         <f aca="false">IF(D72="","",D72/60)</f>
         <v/>
       </c>
-      <c r="F72" s="10"/>
-    </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="9"/>
-      <c r="B73" s="10"/>
-      <c r="C73" s="10"/>
-      <c r="D73" s="11"/>
-      <c r="E73" s="12" t="str">
+      <c r="F72" s="11"/>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A73" s="10"/>
+      <c r="B73" s="11"/>
+      <c r="C73" s="11"/>
+      <c r="D73" s="12"/>
+      <c r="E73" s="13" t="str">
         <f aca="false">IF(D73="","",D73/60)</f>
         <v/>
       </c>
-      <c r="F73" s="10"/>
-    </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="9"/>
-      <c r="B74" s="10"/>
-      <c r="C74" s="10"/>
-      <c r="D74" s="11"/>
-      <c r="E74" s="12" t="str">
+      <c r="F73" s="11"/>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A74" s="10"/>
+      <c r="B74" s="11"/>
+      <c r="C74" s="11"/>
+      <c r="D74" s="12"/>
+      <c r="E74" s="13" t="str">
         <f aca="false">IF(D74="","",D74/60)</f>
         <v/>
       </c>
-      <c r="F74" s="10"/>
-    </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="9"/>
-      <c r="B75" s="10"/>
-      <c r="C75" s="10"/>
-      <c r="D75" s="11"/>
-      <c r="E75" s="12" t="str">
+      <c r="F74" s="11"/>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A75" s="10"/>
+      <c r="B75" s="11"/>
+      <c r="C75" s="11"/>
+      <c r="D75" s="12"/>
+      <c r="E75" s="13" t="str">
         <f aca="false">IF(D75="","",D75/60)</f>
         <v/>
       </c>
-      <c r="F75" s="10"/>
-    </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="9"/>
-      <c r="B76" s="10"/>
-      <c r="C76" s="10"/>
-      <c r="D76" s="11"/>
-      <c r="E76" s="12" t="str">
+      <c r="F75" s="11"/>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A76" s="10"/>
+      <c r="B76" s="11"/>
+      <c r="C76" s="11"/>
+      <c r="D76" s="12"/>
+      <c r="E76" s="13" t="str">
         <f aca="false">IF(D76="","",D76/60)</f>
         <v/>
       </c>
-      <c r="F76" s="10"/>
-    </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="9"/>
-      <c r="B77" s="10"/>
-      <c r="C77" s="10"/>
-      <c r="D77" s="11"/>
-      <c r="E77" s="12" t="str">
+      <c r="F76" s="11"/>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A77" s="10"/>
+      <c r="B77" s="11"/>
+      <c r="C77" s="11"/>
+      <c r="D77" s="12"/>
+      <c r="E77" s="13" t="str">
         <f aca="false">IF(D77="","",D77/60)</f>
         <v/>
       </c>
-      <c r="F77" s="10"/>
-    </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="9"/>
-      <c r="B78" s="10"/>
-      <c r="C78" s="10"/>
-      <c r="D78" s="11"/>
-      <c r="E78" s="12" t="str">
+      <c r="F77" s="11"/>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A78" s="10"/>
+      <c r="B78" s="11"/>
+      <c r="C78" s="11"/>
+      <c r="D78" s="12"/>
+      <c r="E78" s="13" t="str">
         <f aca="false">IF(D78="","",D78/60)</f>
         <v/>
       </c>
-      <c r="F78" s="10"/>
-    </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="9"/>
-      <c r="B79" s="10"/>
-      <c r="C79" s="10"/>
-      <c r="D79" s="11"/>
-      <c r="E79" s="12" t="str">
+      <c r="F78" s="11"/>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A79" s="10"/>
+      <c r="B79" s="11"/>
+      <c r="C79" s="11"/>
+      <c r="D79" s="12"/>
+      <c r="E79" s="13" t="str">
         <f aca="false">IF(D79="","",D79/60)</f>
         <v/>
       </c>
-      <c r="F79" s="10"/>
-    </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="9"/>
-      <c r="B80" s="10"/>
-      <c r="C80" s="10"/>
-      <c r="D80" s="11"/>
-      <c r="E80" s="12" t="str">
+      <c r="F79" s="11"/>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A80" s="10"/>
+      <c r="B80" s="11"/>
+      <c r="C80" s="11"/>
+      <c r="D80" s="12"/>
+      <c r="E80" s="13" t="str">
         <f aca="false">IF(D80="","",D80/60)</f>
         <v/>
       </c>
-      <c r="F80" s="10"/>
-    </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="9"/>
-      <c r="B81" s="10"/>
-      <c r="C81" s="10"/>
-      <c r="D81" s="11"/>
-      <c r="E81" s="12" t="str">
+      <c r="F80" s="11"/>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A81" s="10"/>
+      <c r="B81" s="11"/>
+      <c r="C81" s="11"/>
+      <c r="D81" s="12"/>
+      <c r="E81" s="13" t="str">
         <f aca="false">IF(D81="","",D81/60)</f>
         <v/>
       </c>
-      <c r="F81" s="10"/>
-    </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="9"/>
-      <c r="B82" s="10"/>
-      <c r="C82" s="10"/>
-      <c r="D82" s="11"/>
-      <c r="E82" s="12" t="str">
+      <c r="F81" s="11"/>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A82" s="10"/>
+      <c r="B82" s="11"/>
+      <c r="C82" s="11"/>
+      <c r="D82" s="12"/>
+      <c r="E82" s="13" t="str">
         <f aca="false">IF(D82="","",D82/60)</f>
         <v/>
       </c>
-      <c r="F82" s="10"/>
-    </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="9"/>
-      <c r="B83" s="10"/>
-      <c r="C83" s="10"/>
-      <c r="D83" s="11"/>
-      <c r="E83" s="12" t="str">
+      <c r="F82" s="11"/>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A83" s="10"/>
+      <c r="B83" s="11"/>
+      <c r="C83" s="11"/>
+      <c r="D83" s="12"/>
+      <c r="E83" s="13" t="str">
         <f aca="false">IF(D83="","",D83/60)</f>
         <v/>
       </c>
-      <c r="F83" s="10"/>
-    </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="9"/>
-      <c r="B84" s="10"/>
-      <c r="C84" s="10"/>
-      <c r="D84" s="11"/>
-      <c r="E84" s="12" t="str">
+      <c r="F83" s="11"/>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A84" s="10"/>
+      <c r="B84" s="11"/>
+      <c r="C84" s="11"/>
+      <c r="D84" s="12"/>
+      <c r="E84" s="13" t="str">
         <f aca="false">IF(D84="","",D84/60)</f>
         <v/>
       </c>
-      <c r="F84" s="10"/>
-    </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="9"/>
-      <c r="B85" s="10"/>
-      <c r="C85" s="10"/>
-      <c r="D85" s="11"/>
-      <c r="E85" s="12" t="str">
+      <c r="F84" s="11"/>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A85" s="10"/>
+      <c r="B85" s="11"/>
+      <c r="C85" s="11"/>
+      <c r="D85" s="12"/>
+      <c r="E85" s="13" t="str">
         <f aca="false">IF(D85="","",D85/60)</f>
         <v/>
       </c>
-      <c r="F85" s="10"/>
-    </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="9"/>
-      <c r="B86" s="10"/>
-      <c r="C86" s="10"/>
-      <c r="D86" s="11"/>
-      <c r="E86" s="12" t="str">
+      <c r="F85" s="11"/>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A86" s="10"/>
+      <c r="B86" s="11"/>
+      <c r="C86" s="11"/>
+      <c r="D86" s="12"/>
+      <c r="E86" s="13" t="str">
         <f aca="false">IF(D86="","",D86/60)</f>
         <v/>
       </c>
-      <c r="F86" s="10"/>
-    </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="9"/>
-      <c r="B87" s="10"/>
-      <c r="C87" s="10"/>
-      <c r="D87" s="11"/>
-      <c r="E87" s="12" t="str">
+      <c r="F86" s="11"/>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A87" s="10"/>
+      <c r="B87" s="11"/>
+      <c r="C87" s="11"/>
+      <c r="D87" s="12"/>
+      <c r="E87" s="13" t="str">
         <f aca="false">IF(D87="","",D87/60)</f>
         <v/>
       </c>
-      <c r="F87" s="10"/>
-    </row>
-    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="9"/>
-      <c r="B88" s="10"/>
-      <c r="C88" s="10"/>
-      <c r="D88" s="11"/>
-      <c r="E88" s="12" t="str">
+      <c r="F87" s="11"/>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A88" s="10"/>
+      <c r="B88" s="11"/>
+      <c r="C88" s="11"/>
+      <c r="D88" s="12"/>
+      <c r="E88" s="13" t="str">
         <f aca="false">IF(D88="","",D88/60)</f>
         <v/>
       </c>
-      <c r="F88" s="10"/>
-    </row>
-    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="9"/>
-      <c r="B89" s="10"/>
-      <c r="C89" s="10"/>
-      <c r="D89" s="11"/>
-      <c r="E89" s="12" t="str">
+      <c r="F88" s="11"/>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A89" s="10"/>
+      <c r="B89" s="11"/>
+      <c r="C89" s="11"/>
+      <c r="D89" s="12"/>
+      <c r="E89" s="13" t="str">
         <f aca="false">IF(D89="","",D89/60)</f>
         <v/>
       </c>
-      <c r="F89" s="10"/>
-    </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="9"/>
-      <c r="B90" s="10"/>
-      <c r="C90" s="10"/>
-      <c r="D90" s="11"/>
-      <c r="E90" s="12" t="str">
+      <c r="F89" s="11"/>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A90" s="10"/>
+      <c r="B90" s="11"/>
+      <c r="C90" s="11"/>
+      <c r="D90" s="12"/>
+      <c r="E90" s="13" t="str">
         <f aca="false">IF(D90="","",D90/60)</f>
         <v/>
       </c>
-      <c r="F90" s="10"/>
-    </row>
-    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="9"/>
-      <c r="B91" s="10"/>
-      <c r="C91" s="10"/>
-      <c r="D91" s="11"/>
-      <c r="E91" s="12" t="str">
+      <c r="F90" s="11"/>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A91" s="10"/>
+      <c r="B91" s="11"/>
+      <c r="C91" s="11"/>
+      <c r="D91" s="12"/>
+      <c r="E91" s="13" t="str">
         <f aca="false">IF(D91="","",D91/60)</f>
         <v/>
       </c>
-      <c r="F91" s="10"/>
-    </row>
-    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="9"/>
-      <c r="B92" s="10"/>
-      <c r="C92" s="10"/>
-      <c r="D92" s="11"/>
-      <c r="E92" s="12" t="str">
+      <c r="F91" s="11"/>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A92" s="10"/>
+      <c r="B92" s="11"/>
+      <c r="C92" s="11"/>
+      <c r="D92" s="12"/>
+      <c r="E92" s="13" t="str">
         <f aca="false">IF(D92="","",D92/60)</f>
         <v/>
       </c>
-      <c r="F92" s="10"/>
-    </row>
-    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="9"/>
-      <c r="B93" s="10"/>
-      <c r="C93" s="10"/>
-      <c r="D93" s="11"/>
-      <c r="E93" s="12" t="str">
+      <c r="F92" s="11"/>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A93" s="10"/>
+      <c r="B93" s="11"/>
+      <c r="C93" s="11"/>
+      <c r="D93" s="12"/>
+      <c r="E93" s="13" t="str">
         <f aca="false">IF(D93="","",D93/60)</f>
         <v/>
       </c>
-      <c r="F93" s="10"/>
-    </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="9"/>
-      <c r="B94" s="10"/>
-      <c r="C94" s="10"/>
-      <c r="D94" s="11"/>
-      <c r="E94" s="12" t="str">
+      <c r="F93" s="11"/>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A94" s="10"/>
+      <c r="B94" s="11"/>
+      <c r="C94" s="11"/>
+      <c r="D94" s="12"/>
+      <c r="E94" s="13" t="str">
         <f aca="false">IF(D94="","",D94/60)</f>
         <v/>
       </c>
-      <c r="F94" s="10"/>
-    </row>
-    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="9"/>
-      <c r="B95" s="10"/>
-      <c r="C95" s="10"/>
-      <c r="D95" s="11"/>
-      <c r="E95" s="12" t="str">
+      <c r="F94" s="11"/>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A95" s="10"/>
+      <c r="B95" s="11"/>
+      <c r="C95" s="11"/>
+      <c r="D95" s="12"/>
+      <c r="E95" s="13" t="str">
         <f aca="false">IF(D95="","",D95/60)</f>
         <v/>
       </c>
-      <c r="F95" s="10"/>
-    </row>
-    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="9"/>
-      <c r="B96" s="10"/>
-      <c r="C96" s="10"/>
-      <c r="D96" s="11"/>
-      <c r="E96" s="12" t="str">
+      <c r="F95" s="11"/>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A96" s="10"/>
+      <c r="B96" s="11"/>
+      <c r="C96" s="11"/>
+      <c r="D96" s="12"/>
+      <c r="E96" s="13" t="str">
         <f aca="false">IF(D96="","",D96/60)</f>
         <v/>
       </c>
-      <c r="F96" s="10"/>
-    </row>
-    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="9"/>
-      <c r="B97" s="10"/>
-      <c r="C97" s="10"/>
-      <c r="D97" s="11"/>
-      <c r="E97" s="12" t="str">
+      <c r="F96" s="11"/>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A97" s="10"/>
+      <c r="B97" s="11"/>
+      <c r="C97" s="11"/>
+      <c r="D97" s="12"/>
+      <c r="E97" s="13" t="str">
         <f aca="false">IF(D97="","",D97/60)</f>
         <v/>
       </c>
-      <c r="F97" s="10"/>
-    </row>
-    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="9"/>
-      <c r="B98" s="10"/>
-      <c r="C98" s="10"/>
-      <c r="D98" s="11"/>
-      <c r="E98" s="12" t="str">
+      <c r="F97" s="11"/>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A98" s="10"/>
+      <c r="B98" s="11"/>
+      <c r="C98" s="11"/>
+      <c r="D98" s="12"/>
+      <c r="E98" s="13" t="str">
         <f aca="false">IF(D98="","",D98/60)</f>
         <v/>
       </c>
-      <c r="F98" s="10"/>
-    </row>
-    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="9"/>
-      <c r="B99" s="10"/>
-      <c r="C99" s="10"/>
-      <c r="D99" s="11"/>
-      <c r="E99" s="12" t="str">
+      <c r="F98" s="11"/>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A99" s="10"/>
+      <c r="B99" s="11"/>
+      <c r="C99" s="11"/>
+      <c r="D99" s="12"/>
+      <c r="E99" s="13" t="str">
         <f aca="false">IF(D99="","",D99/60)</f>
         <v/>
       </c>
-      <c r="F99" s="10"/>
-    </row>
-    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="9"/>
-      <c r="B100" s="10"/>
-      <c r="C100" s="10"/>
-      <c r="D100" s="11"/>
-      <c r="E100" s="12" t="str">
+      <c r="F99" s="11"/>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A100" s="10"/>
+      <c r="B100" s="11"/>
+      <c r="C100" s="11"/>
+      <c r="D100" s="12"/>
+      <c r="E100" s="13" t="str">
         <f aca="false">IF(D100="","",D100/60)</f>
         <v/>
       </c>
-      <c r="F100" s="10"/>
-    </row>
-    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="9"/>
-      <c r="B101" s="10"/>
-      <c r="C101" s="10"/>
-      <c r="D101" s="11"/>
-      <c r="E101" s="12" t="str">
+      <c r="F100" s="11"/>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A101" s="10"/>
+      <c r="B101" s="11"/>
+      <c r="C101" s="11"/>
+      <c r="D101" s="12"/>
+      <c r="E101" s="13" t="str">
         <f aca="false">IF(D101="","",D101/60)</f>
         <v/>
       </c>
-      <c r="F101" s="10"/>
-    </row>
-    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="9"/>
-      <c r="B102" s="10"/>
-      <c r="C102" s="10"/>
-      <c r="D102" s="11"/>
-      <c r="E102" s="12" t="str">
+      <c r="F101" s="11"/>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A102" s="10"/>
+      <c r="B102" s="11"/>
+      <c r="C102" s="11"/>
+      <c r="D102" s="12"/>
+      <c r="E102" s="13" t="str">
         <f aca="false">IF(D102="","",D102/60)</f>
         <v/>
       </c>
-      <c r="F102" s="10"/>
-    </row>
-    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="9"/>
-      <c r="B103" s="10"/>
-      <c r="C103" s="10"/>
-      <c r="D103" s="11"/>
-      <c r="E103" s="12" t="str">
+      <c r="F102" s="11"/>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A103" s="10"/>
+      <c r="B103" s="11"/>
+      <c r="C103" s="11"/>
+      <c r="D103" s="12"/>
+      <c r="E103" s="13" t="str">
         <f aca="false">IF(D103="","",D103/60)</f>
         <v/>
       </c>
-      <c r="F103" s="10"/>
-    </row>
-    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A104" s="9"/>
-      <c r="B104" s="10"/>
-      <c r="C104" s="10"/>
-      <c r="D104" s="11"/>
-      <c r="E104" s="12" t="str">
+      <c r="F103" s="11"/>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A104" s="10"/>
+      <c r="B104" s="11"/>
+      <c r="C104" s="11"/>
+      <c r="D104" s="12"/>
+      <c r="E104" s="13" t="str">
         <f aca="false">IF(D104="","",D104/60)</f>
         <v/>
       </c>
-      <c r="F104" s="10"/>
-    </row>
-    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="9"/>
-      <c r="B105" s="10"/>
-      <c r="C105" s="10"/>
-      <c r="D105" s="11"/>
-      <c r="E105" s="12" t="str">
+      <c r="F104" s="11"/>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A105" s="10"/>
+      <c r="B105" s="11"/>
+      <c r="C105" s="11"/>
+      <c r="D105" s="12"/>
+      <c r="E105" s="13" t="str">
         <f aca="false">IF(D105="","",D105/60)</f>
         <v/>
       </c>
-      <c r="F105" s="10"/>
-    </row>
-    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A106" s="9"/>
-      <c r="B106" s="10"/>
-      <c r="C106" s="10"/>
-      <c r="D106" s="11"/>
-      <c r="E106" s="12" t="str">
+      <c r="F105" s="11"/>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A106" s="10"/>
+      <c r="B106" s="11"/>
+      <c r="C106" s="11"/>
+      <c r="D106" s="12"/>
+      <c r="E106" s="13" t="str">
         <f aca="false">IF(D106="","",D106/60)</f>
         <v/>
       </c>
-      <c r="F106" s="10"/>
-    </row>
-    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="9"/>
-      <c r="B107" s="10"/>
-      <c r="C107" s="10"/>
-      <c r="D107" s="11"/>
-      <c r="E107" s="12" t="str">
+      <c r="F106" s="11"/>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A107" s="10"/>
+      <c r="B107" s="11"/>
+      <c r="C107" s="11"/>
+      <c r="D107" s="12"/>
+      <c r="E107" s="13" t="str">
         <f aca="false">IF(D107="","",D107/60)</f>
         <v/>
       </c>
-      <c r="F107" s="10"/>
+      <c r="F107" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2647,7 +2670,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Choose a subcategory from the dropdown list." errorStyle="stop" errorTitle="Invalid subcategory" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C7:C107" type="list">
-      <formula1>Categories!$B$5:$B$22</formula1>
+      <formula1>Categories!$B$5:$B$23</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -2666,509 +2689,521 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
+      <c r="A1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" s="15" t="n">
+      <c r="A2" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="16" t="n">
         <v>46244</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" s="16" t="n">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" s="17" t="n">
         <f aca="false">B4+13</f>
         <v>46257</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="B6" s="16" t="n">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="17" t="n">
         <f aca="true">TODAY()</f>
         <v>46245</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="B7" s="17" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="18" t="n">
         <f aca="false">MAX(B5-B6,0)</f>
         <v>12</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="E9" s="18" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
+    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" s="19" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="19" t="s">
-        <v>32</v>
-      </c>
-      <c r="E10" s="19" t="s">
+      <c r="B10" s="20" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="F10" s="19" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="20" t="s">
+      <c r="F10" s="20" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="21" t="n">
+      <c r="B11" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A11)</f>
-        <v>1.33333333333333</v>
-      </c>
-      <c r="E11" s="22" t="n">
+        <v>3.41666666666667</v>
+      </c>
+      <c r="E11" s="23" t="n">
         <f aca="false">$B$4</f>
         <v>46244</v>
       </c>
-      <c r="F11" s="21" t="n">
+      <c r="F11" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$A$7:$A$107,E11)</f>
         <v>2.58333333333333</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="B12" s="21" t="n">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A12)</f>
         <v>0</v>
       </c>
-      <c r="E12" s="22" t="n">
+      <c r="E12" s="23" t="n">
         <f aca="false">E11+1</f>
         <v>46245</v>
       </c>
-      <c r="F12" s="21" t="n">
+      <c r="F12" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$A$7:$A$107,E12)</f>
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="20" t="s">
-        <v>34</v>
-      </c>
-      <c r="B13" s="21" t="n">
+        <v>2.88333333333333</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A13)</f>
         <v>0</v>
       </c>
-      <c r="E13" s="22" t="n">
+      <c r="E13" s="23" t="n">
         <f aca="false">E12+1</f>
         <v>46246</v>
       </c>
-      <c r="F13" s="21" t="n">
+      <c r="F13" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$A$7:$A$107,E13)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14" s="21" t="n">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="B14" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A14)</f>
         <v>0</v>
       </c>
-      <c r="E14" s="22" t="n">
+      <c r="E14" s="23" t="n">
         <f aca="false">E13+1</f>
         <v>46247</v>
       </c>
-      <c r="F14" s="21" t="n">
+      <c r="F14" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$A$7:$A$107,E14)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="B15" s="21" t="n">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="B15" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A15)</f>
         <v>0</v>
       </c>
-      <c r="E15" s="22" t="n">
+      <c r="E15" s="23" t="n">
         <f aca="false">E14+1</f>
         <v>46248</v>
       </c>
-      <c r="F15" s="21" t="n">
+      <c r="F15" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$A$7:$A$107,E15)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="20" t="s">
-        <v>37</v>
-      </c>
-      <c r="B16" s="21" t="n">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A16)</f>
         <v>0</v>
       </c>
-      <c r="E16" s="22" t="n">
+      <c r="E16" s="23" t="n">
         <f aca="false">E15+1</f>
         <v>46249</v>
       </c>
-      <c r="F16" s="21" t="n">
+      <c r="F16" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$A$7:$A$107,E16)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="20" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="21" t="n">
+      <c r="B17" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A17)</f>
         <v>2.05</v>
       </c>
-      <c r="E17" s="22" t="n">
+      <c r="E17" s="23" t="n">
         <f aca="false">E16+1</f>
         <v>46250</v>
       </c>
-      <c r="F17" s="21" t="n">
+      <c r="F17" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$A$7:$A$107,E17)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="B18" s="24" t="n">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="24" t="s">
+        <v>40</v>
+      </c>
+      <c r="B18" s="25" t="n">
         <f aca="false">SUM(B11:B17)</f>
-        <v>3.38333333333333</v>
-      </c>
-      <c r="E18" s="22" t="n">
+        <v>5.46666666666667</v>
+      </c>
+      <c r="E18" s="23" t="n">
         <f aca="false">E17+1</f>
         <v>46251</v>
       </c>
-      <c r="F18" s="21" t="n">
+      <c r="F18" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$A$7:$A$107,E18)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E19" s="22" t="n">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="E19" s="23" t="n">
         <f aca="false">E18+1</f>
         <v>46252</v>
       </c>
-      <c r="F19" s="21" t="n">
+      <c r="F19" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$A$7:$A$107,E19)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="E20" s="22" t="n">
+    <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="E20" s="23" t="n">
         <f aca="false">E19+1</f>
         <v>46253</v>
       </c>
-      <c r="F20" s="21" t="n">
+      <c r="F20" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$A$7:$A$107,E20)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="19" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="B21" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="C21" s="19" t="s">
-        <v>32</v>
-      </c>
-      <c r="E21" s="22" t="n">
+      <c r="B21" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C21" s="20" t="s">
+        <v>34</v>
+      </c>
+      <c r="E21" s="23" t="n">
         <f aca="false">E20+1</f>
         <v>46254</v>
       </c>
-      <c r="F21" s="21" t="n">
+      <c r="F21" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$A$7:$A$107,E21)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="20" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B22" s="20" t="s">
+      <c r="B22" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="C22" s="21" t="n">
+      <c r="C22" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A22)</f>
         <v>0.75</v>
       </c>
-      <c r="E22" s="22" t="n">
+      <c r="E22" s="23" t="n">
         <f aca="false">E21+1</f>
         <v>46255</v>
       </c>
-      <c r="F22" s="21" t="n">
+      <c r="F22" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$A$7:$A$107,E22)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="20" t="s">
-        <v>41</v>
-      </c>
-      <c r="B23" s="20" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="B23" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="C23" s="21" t="n">
+      <c r="C23" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A23)</f>
         <v>0</v>
       </c>
-      <c r="E23" s="22" t="n">
+      <c r="E23" s="23" t="n">
         <f aca="false">E22+1</f>
         <v>46256</v>
       </c>
-      <c r="F23" s="21" t="n">
+      <c r="F23" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$A$7:$A$107,E23)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="20" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="B24" s="20" t="s">
+      <c r="B24" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="C24" s="21" t="n">
+      <c r="C24" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A24)</f>
         <v>0.0833333333333333</v>
       </c>
-      <c r="E24" s="22" t="n">
+      <c r="E24" s="23" t="n">
         <f aca="false">E23+1</f>
         <v>46257</v>
       </c>
-      <c r="F24" s="21" t="n">
+      <c r="F24" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$A$7:$A$107,E24)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="B25" s="20" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="B25" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="C25" s="21" t="n">
+      <c r="C25" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A25)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="20" t="s">
-        <v>43</v>
-      </c>
-      <c r="B26" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="C26" s="21" t="n">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="B26" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="C26" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A26)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="20" t="s">
-        <v>44</v>
-      </c>
-      <c r="B27" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="C27" s="21" t="n">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="21" t="s">
+        <v>46</v>
+      </c>
+      <c r="B27" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="C27" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A27)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="20" t="s">
-        <v>45</v>
-      </c>
-      <c r="B28" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="C28" s="21" t="n">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="B28" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="C28" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A28)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="20" t="s">
-        <v>46</v>
-      </c>
-      <c r="B29" s="20" t="s">
-        <v>34</v>
-      </c>
-      <c r="C29" s="21" t="n">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="B29" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="C29" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A29)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="20" t="s">
-        <v>47</v>
-      </c>
-      <c r="B30" s="20" t="s">
-        <v>34</v>
-      </c>
-      <c r="C30" s="21" t="n">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="B30" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="C30" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A30)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="20" t="s">
-        <v>48</v>
-      </c>
-      <c r="B31" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="C31" s="21" t="n">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="B31" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="C31" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A31)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="20" t="s">
-        <v>49</v>
-      </c>
-      <c r="B32" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="C32" s="21" t="n">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="B32" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="C32" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A32)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="20" t="s">
-        <v>50</v>
-      </c>
-      <c r="B33" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="C33" s="21" t="n">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="B33" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="C33" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A33)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="20" t="s">
-        <v>51</v>
-      </c>
-      <c r="B34" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="C34" s="21" t="n">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="B34" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="C34" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A34)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="20" t="s">
-        <v>52</v>
-      </c>
-      <c r="B35" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="C35" s="21" t="n">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="B35" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="C35" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A35)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="20" t="s">
-        <v>53</v>
-      </c>
-      <c r="B36" s="20" t="s">
-        <v>37</v>
-      </c>
-      <c r="C36" s="21" t="n">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="B36" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="C36" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A36)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="20" t="s">
-        <v>54</v>
-      </c>
-      <c r="B37" s="20" t="s">
-        <v>37</v>
-      </c>
-      <c r="C37" s="21" t="n">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="B37" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="C37" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A37)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="20" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="B38" s="20" t="s">
+      <c r="B38" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="C38" s="21" t="n">
+      <c r="C38" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A38)</f>
         <v>2.05</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="20" t="s">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B39" s="20" t="s">
+      <c r="B39" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="C39" s="21" t="n">
+      <c r="C39" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A39)</f>
         <v>0.5</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="B40" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="C40" s="22" t="n">
+        <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A40)</f>
+        <v>2.08333333333333</v>
       </c>
     </row>
   </sheetData>
@@ -3192,204 +3227,212 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="30"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="27" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="28" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="28" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="28" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="B8" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" s="21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" s="21" t="s">
+        <v>46</v>
+      </c>
+      <c r="C10" s="21" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11" s="21" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B12" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="C12" s="21" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" s="21" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B14" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="C14" s="21" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="C15" s="21" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B16" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="C16" s="21" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="C17" s="21" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B18" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="C18" s="21" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B19" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="26" t="s">
+      <c r="C19" s="21" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B20" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="27" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="27" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="27" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="20" t="s">
+      <c r="C20" s="21" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B21" s="21" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="21" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B22" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C22" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="20" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="B6" s="20" t="s">
-        <v>41</v>
-      </c>
-      <c r="C6" s="20" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="20" t="s">
-        <v>34</v>
-      </c>
-      <c r="B7" s="20" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" s="20" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="B8" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="C8" s="20" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="B9" s="20" t="s">
-        <v>43</v>
-      </c>
-      <c r="C9" s="20" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="20" t="s">
-        <v>37</v>
-      </c>
-      <c r="B10" s="20" t="s">
-        <v>44</v>
-      </c>
-      <c r="C10" s="20" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="20" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" s="20" t="s">
-        <v>45</v>
-      </c>
-      <c r="C11" s="20" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="20" t="s">
-        <v>46</v>
-      </c>
-      <c r="C12" s="20" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="20" t="s">
-        <v>47</v>
-      </c>
-      <c r="C13" s="20" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="20" t="s">
-        <v>48</v>
-      </c>
-      <c r="C14" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="20" t="s">
-        <v>49</v>
-      </c>
-      <c r="C15" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="20" t="s">
-        <v>50</v>
-      </c>
-      <c r="C16" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="20" t="s">
-        <v>51</v>
-      </c>
-      <c r="C17" s="20" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="20" t="s">
-        <v>52</v>
-      </c>
-      <c r="C18" s="20" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="20" t="s">
-        <v>53</v>
-      </c>
-      <c r="C19" s="20" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="20" t="s">
-        <v>54</v>
-      </c>
-      <c r="C20" s="20" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="20" t="s">
-        <v>15</v>
-      </c>
-      <c r="C21" s="20" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="20" t="s">
-        <v>17</v>
-      </c>
-      <c r="C22" s="20" t="s">
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C23" s="21" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Time tracker logged 15 min to Marketing/Email; today's hike logged (3.7 mi, corrected pace to 20:00/mile); three LinkedIn drafts built from Jackie's own concepts (AI image tells, time framework vs. audit, AI-written contracts) and delivered as md/docx; time-framework draft assigned to Monday 8/24, two drafts left open for a later week
</commit_message>
<xml_diff>
--- a/outputs/time-tracking/business-activity-time-tracker.xlsx
+++ b/outputs/time-tracking/business-activity-time-tracker.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc"/>
+  <fileVersion appName="Calc" lowestEdited="4"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="60">
   <si>
     <t xml:space="preserve">Business Activity Time Tracker</t>
   </si>
@@ -773,7 +773,7 @@
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>3.41666666666667</c:v>
+                  <c:v>3.66666666666667</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -799,11 +799,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="8391556"/>
-        <c:axId val="86258886"/>
+        <c:axId val="21932158"/>
+        <c:axId val="18400528"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="8391556"/>
+        <c:axId val="21932158"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -836,7 +836,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86258886"/>
+        <c:crossAx val="18400528"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -844,7 +844,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="86258886"/>
+        <c:axId val="18400528"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -920,7 +920,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="8391556"/>
+        <c:crossAx val="21932158"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1177,9 +1177,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>305280</xdr:colOff>
+      <xdr:colOff>304920</xdr:colOff>
       <xdr:row>40</xdr:row>
-      <xdr:rowOff>21960</xdr:rowOff>
+      <xdr:rowOff>21600</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1188,7 +1188,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="6673320" y="4952880"/>
-        <a:ext cx="5759280" cy="2879640"/>
+        <a:ext cx="5758920" cy="2879280"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1658,15 +1658,25 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10"/>
-      <c r="B17" s="11"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="13" t="str">
+      <c r="A17" s="10" t="n">
+        <v>46246</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="E17" s="13" t="n">
         <f aca="false">IF(D17="","",D17/60)</f>
-        <v/>
-      </c>
-      <c r="F17" s="11"/>
+        <v>0.25</v>
+      </c>
+      <c r="F17" s="11" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="10"/>
@@ -2742,7 +2752,7 @@
       </c>
       <c r="B6" s="17" t="n">
         <f aca="true">TODAY()</f>
-        <v>46245</v>
+        <v>46246</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2751,7 +2761,7 @@
       </c>
       <c r="B7" s="18" t="n">
         <f aca="false">MAX(B5-B6,0)</f>
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2782,7 +2792,7 @@
       </c>
       <c r="B11" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A11)</f>
-        <v>3.41666666666667</v>
+        <v>3.66666666666667</v>
       </c>
       <c r="E11" s="23" t="n">
         <f aca="false">$B$4</f>
@@ -2824,7 +2834,7 @@
       </c>
       <c r="F13" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$A$7:$A$107,E13)</f>
-        <v>0</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2901,7 +2911,7 @@
       </c>
       <c r="B18" s="25" t="n">
         <f aca="false">SUM(B11:B17)</f>
-        <v>5.46666666666667</v>
+        <v>5.71666666666667</v>
       </c>
       <c r="E18" s="23" t="n">
         <f aca="false">E17+1</f>
@@ -2963,7 +2973,7 @@
       </c>
       <c r="C22" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A22)</f>
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="E22" s="23" t="n">
         <f aca="false">E21+1</f>
@@ -3194,7 +3204,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="21" t="s">
         <v>24</v>
       </c>
@@ -3428,7 +3438,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="21" t="s">
         <v>24</v>
       </c>

</xml_diff>

<commit_message>
Website redesign status reviewed against live Gmail, real sign-off gaps found and memory rebuilt; Diane Leonard catch-up logged with three reminders set and a follow-up drafted (her rewrite taught new writing-voice patterns around third-party health details); Work With Me page built, reviewed across several rounds catching real scope and voice issues, and shipped as matching copy doc and HTML mockup
</commit_message>
<xml_diff>
--- a/outputs/time-tracking/business-activity-time-tracker.xlsx
+++ b/outputs/time-tracking/business-activity-time-tracker.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="62">
   <si>
     <t xml:space="preserve">Business Activity Time Tracker</t>
   </si>
@@ -100,6 +100,12 @@
   </si>
   <si>
     <t xml:space="preserve">Blog post review/edit, built out and published in WordPress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Client reconnection marketing - Diane Leonard catch-up notes, meeting log, follow-up email draft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LinkedIn marketing</t>
   </si>
   <si>
     <t xml:space="preserve">Time Tracking Summary</t>
@@ -773,7 +779,7 @@
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>3.66666666666667</c:v>
+                  <c:v>4.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -799,11 +805,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="21932158"/>
-        <c:axId val="18400528"/>
+        <c:axId val="51169628"/>
+        <c:axId val="95438136"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="21932158"/>
+        <c:axId val="51169628"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -836,7 +842,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="18400528"/>
+        <c:crossAx val="95438136"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -844,7 +850,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="18400528"/>
+        <c:axId val="95438136"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -920,7 +926,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="21932158"/>
+        <c:crossAx val="51169628"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1177,9 +1183,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>304920</xdr:colOff>
+      <xdr:colOff>304560</xdr:colOff>
       <xdr:row>40</xdr:row>
-      <xdr:rowOff>21600</xdr:rowOff>
+      <xdr:rowOff>21240</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1188,7 +1194,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="6673320" y="4952880"/>
-        <a:ext cx="5758920" cy="2879280"/>
+        <a:ext cx="5758560" cy="2878920"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1679,26 +1685,46 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10"/>
-      <c r="B18" s="11"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="13" t="str">
+      <c r="A18" s="10" t="n">
+        <v>46246</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D18" s="12" t="n">
+        <v>45</v>
+      </c>
+      <c r="E18" s="13" t="n">
         <f aca="false">IF(D18="","",D18/60)</f>
-        <v/>
-      </c>
-      <c r="F18" s="11"/>
+        <v>0.75</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10"/>
-      <c r="B19" s="11"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="13" t="str">
+      <c r="A19" s="10" t="n">
+        <v>46246</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="E19" s="13" t="n">
         <f aca="false">IF(D19="","",D19/60)</f>
-        <v/>
-      </c>
-      <c r="F19" s="11"/>
+        <v>0.0833333333333333</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="10"/>
@@ -2711,7 +2737,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2721,7 +2747,7 @@
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B2" s="14"/>
       <c r="C2" s="14"/>
@@ -2731,7 +2757,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B4" s="16" t="n">
         <v>46244</v>
@@ -2739,7 +2765,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B5" s="17" t="n">
         <f aca="false">B4+13</f>
@@ -2748,7 +2774,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B6" s="17" t="n">
         <f aca="true">TODAY()</f>
@@ -2757,7 +2783,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B7" s="18" t="n">
         <f aca="false">MAX(B5-B6,0)</f>
@@ -2766,10 +2792,10 @@
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2777,13 +2803,13 @@
         <v>4</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>3</v>
       </c>
       <c r="F10" s="20" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2792,7 +2818,7 @@
       </c>
       <c r="B11" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A11)</f>
-        <v>3.66666666666667</v>
+        <v>4.5</v>
       </c>
       <c r="E11" s="23" t="n">
         <f aca="false">$B$4</f>
@@ -2805,7 +2831,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="21" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B12" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A12)</f>
@@ -2822,7 +2848,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="21" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B13" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A13)</f>
@@ -2834,12 +2860,12 @@
       </c>
       <c r="F13" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$A$7:$A$107,E13)</f>
-        <v>0.25</v>
+        <v>1.08333333333333</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="21" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B14" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A14)</f>
@@ -2856,7 +2882,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="21" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B15" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A15)</f>
@@ -2873,7 +2899,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="21" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B16" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A16)</f>
@@ -2907,11 +2933,11 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="24" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B18" s="25" t="n">
         <f aca="false">SUM(B11:B17)</f>
-        <v>5.71666666666667</v>
+        <v>6.55</v>
       </c>
       <c r="E18" s="23" t="n">
         <f aca="false">E17+1</f>
@@ -2934,7 +2960,7 @@
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="19" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E20" s="23" t="n">
         <f aca="false">E19+1</f>
@@ -2950,10 +2976,10 @@
         <v>5</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C21" s="20" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E21" s="23" t="n">
         <f aca="false">E20+1</f>
@@ -2986,7 +3012,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="21" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B23" s="21" t="s">
         <v>9</v>
@@ -3013,7 +3039,7 @@
       </c>
       <c r="C24" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A24)</f>
-        <v>0.0833333333333333</v>
+        <v>0.166666666666667</v>
       </c>
       <c r="E24" s="23" t="n">
         <f aca="false">E23+1</f>
@@ -3026,7 +3052,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="21" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B25" s="21" t="s">
         <v>9</v>
@@ -3038,10 +3064,10 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="21" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C26" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A26)</f>
@@ -3050,10 +3076,10 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="21" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C27" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A27)</f>
@@ -3062,10 +3088,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="21" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C28" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A28)</f>
@@ -3074,10 +3100,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="21" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C29" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A29)</f>
@@ -3086,10 +3112,10 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="21" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C30" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A30)</f>
@@ -3098,10 +3124,10 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="21" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C31" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A31)</f>
@@ -3110,10 +3136,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="21" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B32" s="21" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C32" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A32)</f>
@@ -3122,10 +3148,10 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="21" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C33" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A33)</f>
@@ -3134,10 +3160,10 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="21" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B34" s="21" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C34" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A34)</f>
@@ -3146,10 +3172,10 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="21" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B35" s="21" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C35" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A35)</f>
@@ -3158,10 +3184,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="21" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B36" s="21" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C36" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A36)</f>
@@ -3170,10 +3196,10 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="21" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B37" s="21" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C37" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A37)</f>
@@ -3201,7 +3227,7 @@
       </c>
       <c r="C39" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A39)</f>
-        <v>0.5</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3247,7 +3273,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="26" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B1" s="26"/>
       <c r="C1" s="26"/>
@@ -3257,7 +3283,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="27" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B2" s="27"/>
       <c r="C2" s="27"/>
@@ -3270,7 +3296,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="28" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3286,10 +3312,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="21" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C6" s="21" t="s">
         <v>9</v>
@@ -3297,7 +3323,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="21" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B7" s="21" t="s">
         <v>10</v>
@@ -3308,10 +3334,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="21" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C8" s="21" t="s">
         <v>9</v>
@@ -3319,24 +3345,24 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="21" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="21" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3344,82 +3370,82 @@
         <v>14</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="21" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C12" s="21" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="21" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C13" s="21" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="21" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C14" s="21" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="21" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C15" s="21" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="21" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="21" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="21" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C18" s="21" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="21" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C19" s="21" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="21" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Work With Me page deployed to staging as a new page, WP deploy mechanics (theme-override + button-fix CSS, HTML-comment-stripping gotcha) discovered and documented; Brooke Billingsley client quote mocked up and added between the two tracks, quote marks removed on request; draft-email style check compared Gmail inbox-reply drafts (HubSpot Active Engagers found unchanged) and logged new voice patterns to memory; Day B strength session and hill warmup logged after resolving voice-dictation ambiguities with Jackie directly
</commit_message>
<xml_diff>
--- a/outputs/time-tracking/business-activity-time-tracker.xlsx
+++ b/outputs/time-tracking/business-activity-time-tracker.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="64">
   <si>
     <t xml:space="preserve">Business Activity Time Tracker</t>
   </si>
@@ -106,6 +106,12 @@
   </si>
   <si>
     <t xml:space="preserve">LinkedIn marketing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Website Design (Marketing)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Work With Me page copy build, review rounds, and HTML mockup</t>
   </si>
   <si>
     <t xml:space="preserve">Time Tracking Summary</t>
@@ -779,7 +785,7 @@
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>4.5</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -805,11 +811,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="51169628"/>
-        <c:axId val="95438136"/>
+        <c:axId val="95974912"/>
+        <c:axId val="118022"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="51169628"/>
+        <c:axId val="95974912"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -842,7 +848,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="95438136"/>
+        <c:crossAx val="118022"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -850,7 +856,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="95438136"/>
+        <c:axId val="118022"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -926,7 +932,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="51169628"/>
+        <c:crossAx val="95974912"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1183,9 +1189,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>304560</xdr:colOff>
+      <xdr:colOff>304200</xdr:colOff>
       <xdr:row>40</xdr:row>
-      <xdr:rowOff>21240</xdr:rowOff>
+      <xdr:rowOff>20880</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1194,7 +1200,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="6673320" y="4952880"/>
-        <a:ext cx="5758560" cy="2878920"/>
+        <a:ext cx="5758200" cy="2878560"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1727,15 +1733,25 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10"/>
-      <c r="B20" s="11"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="13" t="str">
+      <c r="A20" s="10" t="n">
+        <v>46246</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="D20" s="12" t="n">
+        <v>90</v>
+      </c>
+      <c r="E20" s="13" t="n">
         <f aca="false">IF(D20="","",D20/60)</f>
-        <v/>
-      </c>
-      <c r="F20" s="11"/>
+        <v>1.5</v>
+      </c>
+      <c r="F20" s="11" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="10"/>
@@ -2706,7 +2722,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Choose a subcategory from the dropdown list." errorStyle="stop" errorTitle="Invalid subcategory" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C7:C107" type="list">
-      <formula1>Categories!$B$5:$B$23</formula1>
+      <formula1>Categories!$B$5:$B$24</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -2737,7 +2753,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2747,7 +2763,7 @@
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B2" s="14"/>
       <c r="C2" s="14"/>
@@ -2757,7 +2773,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B4" s="16" t="n">
         <v>46244</v>
@@ -2765,7 +2781,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B5" s="17" t="n">
         <f aca="false">B4+13</f>
@@ -2774,7 +2790,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B6" s="17" t="n">
         <f aca="true">TODAY()</f>
@@ -2783,7 +2799,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B7" s="18" t="n">
         <f aca="false">MAX(B5-B6,0)</f>
@@ -2792,10 +2808,10 @@
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2803,13 +2819,13 @@
         <v>4</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>3</v>
       </c>
       <c r="F10" s="20" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2818,7 +2834,7 @@
       </c>
       <c r="B11" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A11)</f>
-        <v>4.5</v>
+        <v>6</v>
       </c>
       <c r="E11" s="23" t="n">
         <f aca="false">$B$4</f>
@@ -2831,7 +2847,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="21" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B12" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A12)</f>
@@ -2848,7 +2864,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="21" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B13" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A13)</f>
@@ -2860,12 +2876,12 @@
       </c>
       <c r="F13" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$A$7:$A$107,E13)</f>
-        <v>1.08333333333333</v>
+        <v>2.58333333333333</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="21" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B14" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A14)</f>
@@ -2882,7 +2898,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="21" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B15" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A15)</f>
@@ -2899,7 +2915,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="21" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B16" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$B$7:$B$107,A16)</f>
@@ -2933,11 +2949,11 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="24" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B18" s="25" t="n">
         <f aca="false">SUM(B11:B17)</f>
-        <v>6.55</v>
+        <v>8.05</v>
       </c>
       <c r="E18" s="23" t="n">
         <f aca="false">E17+1</f>
@@ -2960,7 +2976,7 @@
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="19" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E20" s="23" t="n">
         <f aca="false">E19+1</f>
@@ -2976,10 +2992,10 @@
         <v>5</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C21" s="20" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E21" s="23" t="n">
         <f aca="false">E20+1</f>
@@ -3012,7 +3028,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="21" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B23" s="21" t="s">
         <v>9</v>
@@ -3052,7 +3068,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="21" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B25" s="21" t="s">
         <v>9</v>
@@ -3064,10 +3080,10 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="21" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C26" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A26)</f>
@@ -3076,10 +3092,10 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="21" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C27" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A27)</f>
@@ -3088,10 +3104,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="21" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C28" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A28)</f>
@@ -3100,10 +3116,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="21" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C29" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A29)</f>
@@ -3112,10 +3128,10 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="21" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C30" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A30)</f>
@@ -3124,10 +3140,10 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="21" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C31" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A31)</f>
@@ -3136,10 +3152,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="21" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B32" s="21" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C32" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A32)</f>
@@ -3148,10 +3164,10 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="21" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C33" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A33)</f>
@@ -3160,10 +3176,10 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="21" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B34" s="21" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C34" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A34)</f>
@@ -3172,10 +3188,10 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="21" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B35" s="21" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C35" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A35)</f>
@@ -3184,10 +3200,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="21" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B36" s="21" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C36" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A36)</f>
@@ -3196,10 +3212,10 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="21" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B37" s="21" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C37" s="22" t="n">
         <f aca="false">SUMIFS('Time Log'!$E$7:$E$107,'Time Log'!$C$7:$C$107,A37)</f>
@@ -3263,7 +3279,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28"/>
@@ -3273,7 +3289,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="26" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B1" s="26"/>
       <c r="C1" s="26"/>
@@ -3283,7 +3299,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="27" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B2" s="27"/>
       <c r="C2" s="27"/>
@@ -3296,7 +3312,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="28" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3312,10 +3328,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="21" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C6" s="21" t="s">
         <v>9</v>
@@ -3323,7 +3339,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="21" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B7" s="21" t="s">
         <v>10</v>
@@ -3334,10 +3350,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="21" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C8" s="21" t="s">
         <v>9</v>
@@ -3345,24 +3361,24 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="21" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="21" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3370,82 +3386,82 @@
         <v>14</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="21" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C12" s="21" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="21" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C13" s="21" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="21" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C14" s="21" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="21" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C15" s="21" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="21" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="21" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="21" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C18" s="21" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="21" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C19" s="21" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="21" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3469,6 +3485,14 @@
         <v>24</v>
       </c>
       <c r="C23" s="21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>